<commit_message>
pass process DUT and GER item correction
</commit_message>
<xml_diff>
--- a/Scales-pas/PASS-process/Petri-Romão_2024_PASS-process_DUT.xlsx
+++ b/Scales-pas/PASS-process/Petri-Romão_2024_PASS-process_DUT.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28429"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="P:\Papoula\Research\PHD\Projects\Organising all questionnaires\PAS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{2A581F5E-D77E-44A4-84D4-AAF63304B5BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{96CC9651-46BB-46E7-B90B-4FA46B4499A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-78" yWindow="0" windowWidth="8796" windowHeight="10878" xr2:uid="{2243D91A-F1AD-4BAA-BD82-86E6A3DB83B8}"/>
+    <workbookView xWindow="42465" yWindow="-16320" windowWidth="29040" windowHeight="16440" xr2:uid="{2243D91A-F1AD-4BAA-BD82-86E6A3DB83B8}"/>
   </bookViews>
   <sheets>
     <sheet name="PASS-process DUT" sheetId="1" r:id="rId1"/>
@@ -48,9 +48,6 @@
     <t>Ik bedenk me dat ik moet aanvaarden dat mij dit is overkomen.</t>
   </si>
   <si>
-    <t>Ik denk aan leukere dingen dan wat ik heb meegemaakt.</t>
-  </si>
-  <si>
     <t>Ik bedenk me dat ik het moet accepteren.</t>
   </si>
   <si>
@@ -73,6 +70,9 @@
   </si>
   <si>
     <t>1 = (bijna) nooit 2 = soms 3 = regelmatig 4 = vaak 5 = (bijna) altijd</t>
+  </si>
+  <si>
+    <t>Ik denk dat ik als persoon ‘sterker’ word door de situatie.</t>
   </si>
 </sst>
 </file>
@@ -193,15 +193,6 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
@@ -213,6 +204,15 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -535,181 +535,187 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="153.75" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A1" s="5" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="8" t="s">
+      <c r="B1" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="8"/>
-      <c r="D1" s="8"/>
-      <c r="E1" s="8"/>
-      <c r="F1" s="8"/>
-      <c r="G1" s="8"/>
-      <c r="H1" s="8"/>
+      <c r="C1" s="5"/>
+      <c r="D1" s="5"/>
+      <c r="E1" s="5"/>
+      <c r="F1" s="5"/>
+      <c r="G1" s="5"/>
+      <c r="H1" s="5"/>
     </row>
     <row r="2" spans="1:8" ht="105" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A2" s="6"/>
+      <c r="A2" s="3"/>
       <c r="B2" s="1">
         <v>1</v>
       </c>
-      <c r="C2" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="D2" s="3"/>
-      <c r="E2" s="3"/>
-      <c r="F2" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="G2" s="3"/>
-      <c r="H2" s="3"/>
+      <c r="C2" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="D2" s="7"/>
+      <c r="E2" s="7"/>
+      <c r="F2" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="G2" s="7"/>
+      <c r="H2" s="7"/>
     </row>
     <row r="3" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A3" s="6"/>
+      <c r="A3" s="3"/>
       <c r="B3" s="1">
         <v>2</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="C3" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="D3" s="3"/>
-      <c r="E3" s="3"/>
-      <c r="F3" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="G3" s="3"/>
-      <c r="H3" s="3"/>
+      <c r="D3" s="7"/>
+      <c r="E3" s="7"/>
+      <c r="F3" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3" s="7"/>
+      <c r="H3" s="7"/>
     </row>
     <row r="4" spans="1:8" ht="85.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A4" s="6"/>
+      <c r="A4" s="3"/>
       <c r="B4" s="1">
         <v>3</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="C4" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="D4" s="3"/>
-      <c r="E4" s="4"/>
-      <c r="F4" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="G4" s="3"/>
-      <c r="H4" s="3"/>
+      <c r="D4" s="7"/>
+      <c r="E4" s="8"/>
+      <c r="F4" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="G4" s="7"/>
+      <c r="H4" s="7"/>
     </row>
     <row r="5" spans="1:8" ht="85.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A5" s="6"/>
+      <c r="A5" s="3"/>
       <c r="B5" s="1">
         <v>4</v>
       </c>
-      <c r="C5" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="D5" s="3"/>
-      <c r="E5" s="4"/>
-      <c r="F5" s="2" t="s">
+      <c r="C5" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="G5" s="3"/>
-      <c r="H5" s="3"/>
+      <c r="D5" s="7"/>
+      <c r="E5" s="8"/>
+      <c r="F5" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="G5" s="7"/>
+      <c r="H5" s="7"/>
     </row>
     <row r="6" spans="1:8" ht="85.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A6" s="6"/>
+      <c r="A6" s="3"/>
       <c r="B6" s="1">
         <v>5</v>
       </c>
-      <c r="C6" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="D6" s="3"/>
-      <c r="E6" s="4"/>
-      <c r="F6" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="G6" s="3"/>
-      <c r="H6" s="3"/>
+      <c r="C6" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="D6" s="7"/>
+      <c r="E6" s="8"/>
+      <c r="F6" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="G6" s="7"/>
+      <c r="H6" s="7"/>
     </row>
     <row r="7" spans="1:8" ht="85.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A7" s="6"/>
+      <c r="A7" s="3"/>
       <c r="B7" s="1">
         <v>6</v>
       </c>
-      <c r="C7" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="D7" s="3"/>
-      <c r="E7" s="4"/>
-      <c r="F7" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="G7" s="3"/>
-      <c r="H7" s="3"/>
+      <c r="C7" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="D7" s="7"/>
+      <c r="E7" s="8"/>
+      <c r="F7" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="G7" s="7"/>
+      <c r="H7" s="7"/>
     </row>
     <row r="8" spans="1:8" ht="85.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A8" s="6"/>
+      <c r="A8" s="3"/>
       <c r="B8" s="1">
         <v>7</v>
       </c>
-      <c r="C8" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="D8" s="3"/>
-      <c r="E8" s="4"/>
-      <c r="F8" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="G8" s="3"/>
-      <c r="H8" s="3"/>
+      <c r="C8" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="D8" s="7"/>
+      <c r="E8" s="8"/>
+      <c r="F8" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="G8" s="7"/>
+      <c r="H8" s="7"/>
     </row>
     <row r="9" spans="1:8" ht="85.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A9" s="6"/>
+      <c r="A9" s="3"/>
       <c r="B9" s="1">
         <v>8</v>
       </c>
-      <c r="C9" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="D9" s="3"/>
-      <c r="E9" s="4"/>
-      <c r="F9" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="G9" s="3"/>
-      <c r="H9" s="3"/>
+      <c r="C9" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="D9" s="7"/>
+      <c r="E9" s="8"/>
+      <c r="F9" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="G9" s="7"/>
+      <c r="H9" s="7"/>
     </row>
     <row r="10" spans="1:8" ht="85.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A10" s="6"/>
+      <c r="A10" s="3"/>
       <c r="B10" s="1">
         <v>9</v>
       </c>
-      <c r="C10" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="D10" s="3"/>
-      <c r="E10" s="4"/>
-      <c r="F10" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="G10" s="3"/>
-      <c r="H10" s="3"/>
+      <c r="C10" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="D10" s="7"/>
+      <c r="E10" s="8"/>
+      <c r="F10" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="G10" s="7"/>
+      <c r="H10" s="7"/>
     </row>
     <row r="11" spans="1:8" ht="85.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A11" s="7"/>
+      <c r="A11" s="4"/>
       <c r="B11" s="1">
         <v>10</v>
       </c>
-      <c r="C11" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="D11" s="3"/>
-      <c r="E11" s="4"/>
-      <c r="F11" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="G11" s="3"/>
-      <c r="H11" s="3"/>
+      <c r="C11" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="D11" s="7"/>
+      <c r="E11" s="8"/>
+      <c r="F11" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="G11" s="7"/>
+      <c r="H11" s="7"/>
     </row>
   </sheetData>
   <mergeCells count="22">
+    <mergeCell ref="C4:E4"/>
+    <mergeCell ref="F7:H7"/>
+    <mergeCell ref="C5:E5"/>
+    <mergeCell ref="C6:E6"/>
+    <mergeCell ref="F5:H5"/>
+    <mergeCell ref="F6:H6"/>
     <mergeCell ref="A1:A11"/>
     <mergeCell ref="B1:H1"/>
     <mergeCell ref="C11:E11"/>
@@ -726,12 +732,6 @@
     <mergeCell ref="F2:H2"/>
     <mergeCell ref="C3:E3"/>
     <mergeCell ref="F3:H3"/>
-    <mergeCell ref="C4:E4"/>
-    <mergeCell ref="F7:H7"/>
-    <mergeCell ref="C5:E5"/>
-    <mergeCell ref="C6:E6"/>
-    <mergeCell ref="F5:H5"/>
-    <mergeCell ref="F6:H6"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>